<commit_message>
feat: learned equipment classification from registry descriptions (94% validated)
</commit_message>
<xml_diff>
--- a/tests/fixtures/compiler-extoreg.xlsx
+++ b/tests/fixtures/compiler-extoreg.xlsx
@@ -409,7 +409,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:J7"/>
+  <dimension ref="A1:K7"/>
   <sheetData>
     <row r="1">
       <c r="A1" s="2" t="str">
@@ -437,9 +437,12 @@
         <v>Equipment Description</v>
       </c>
       <c r="I1" s="2" t="str">
+        <v>Equipment Classification</v>
+      </c>
+      <c r="J1" s="2" t="str">
         <v>Closest Parent</v>
       </c>
-      <c r="J1" s="2" t="str">
+      <c r="K1" s="2" t="str">
         <v>Item Master Unique Identifier</v>
       </c>
     </row>
@@ -469,9 +472,12 @@
         <v>Remote IO panel</v>
       </c>
       <c r="I2" s="2" t="str">
+        <v>RIO</v>
+      </c>
+      <c r="J2" s="2" t="str">
         <v>650 FMS Network</v>
       </c>
-      <c r="J2" s="2" t="str">
+      <c r="K2" s="2" t="str">
         <v>CA_NB_IC_RIO</v>
       </c>
     </row>
@@ -501,9 +507,12 @@
         <v>Air handler</v>
       </c>
       <c r="I3" s="2" t="str">
+        <v>AHU</v>
+      </c>
+      <c r="J3" s="2" t="str">
         <v>2201 Screening</v>
       </c>
-      <c r="J3" s="2" t="str">
+      <c r="K3" s="2" t="str">
         <v>VF_MECH_AHU</v>
       </c>
     </row>
@@ -533,9 +542,12 @@
         <v>Supply fan motor</v>
       </c>
       <c r="I4" s="2" t="str">
+        <v>MTR</v>
+      </c>
+      <c r="J4" s="2" t="str">
         <v>X-AHU-9</v>
       </c>
-      <c r="J4" s="2" t="str">
+      <c r="K4" s="2" t="str">
         <v>VF_MECH_FAN</v>
       </c>
     </row>
@@ -562,12 +574,15 @@
         <v>X-M2</v>
       </c>
       <c r="H5" s="2" t="str">
-        <v>Supply pump</v>
+        <v>Supply fan motor</v>
       </c>
       <c r="I5" s="2" t="str">
+        <v>MTR</v>
+      </c>
+      <c r="J5" s="2" t="str">
         <v>X-AHU-9</v>
       </c>
-      <c r="J5" s="2" t="str">
+      <c r="K5" s="2" t="str">
         <v>VF_MECH_PUMP</v>
       </c>
     </row>
@@ -597,9 +612,12 @@
         <v>Makeup pump</v>
       </c>
       <c r="I6" s="2" t="str">
+        <v>PMP</v>
+      </c>
+      <c r="J6" s="2" t="str">
         <v>241 UPW Makeup</v>
       </c>
-      <c r="J6" s="2" t="str">
+      <c r="K6" s="2" t="str">
         <v>CA_NB_EL_MV_GEAR</v>
       </c>
     </row>
@@ -629,15 +647,18 @@
         <v>Isolation valve</v>
       </c>
       <c r="I7" s="2" t="str">
+        <v>XV</v>
+      </c>
+      <c r="J7" s="2" t="str">
         <v>266 HFW Treatment</v>
       </c>
-      <c r="J7" s="2" t="str">
+      <c r="K7" s="2" t="str">
         <v>VF_Blank</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:J7"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:K7"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
feat: description-role + number-nomenclature nesting proposals (propose-don't-assume)
</commit_message>
<xml_diff>
--- a/tests/fixtures/compiler-extoreg.xlsx
+++ b/tests/fixtures/compiler-extoreg.xlsx
@@ -409,7 +409,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:K7"/>
+  <dimension ref="A1:K17"/>
   <sheetData>
     <row r="1">
       <c r="A1" s="2" t="str">
@@ -623,42 +623,392 @@
     </row>
     <row r="7">
       <c r="A7" s="2" t="str">
+        <v>E-T0</v>
+      </c>
+      <c r="B7" s="2" t="str">
+        <v>B1</v>
+      </c>
+      <c r="C7" s="2" t="str">
+        <v>B14</v>
+      </c>
+      <c r="D7" s="2" t="str">
+        <v>2201</v>
+      </c>
+      <c r="E7" s="2" t="str">
+        <v>MECHANICAL</v>
+      </c>
+      <c r="F7" s="2" t="str">
+        <v>2201 Screening</v>
+      </c>
+      <c r="G7" s="2" t="str">
+        <v>X-TT-0</v>
+      </c>
+      <c r="H7" s="2" t="str">
+        <v>Temperature transmitter</v>
+      </c>
+      <c r="I7" s="2" t="str">
+        <v>TT</v>
+      </c>
+      <c r="J7" s="2" t="str">
+        <v>X-AHU-9</v>
+      </c>
+      <c r="K7" s="2" t="str">
+        <v>VF_I&amp;C_TRANSMITTER</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="str">
+        <v>E-T1</v>
+      </c>
+      <c r="B8" s="2" t="str">
+        <v>B1</v>
+      </c>
+      <c r="C8" s="2" t="str">
+        <v>B14</v>
+      </c>
+      <c r="D8" s="2" t="str">
+        <v>2201</v>
+      </c>
+      <c r="E8" s="2" t="str">
+        <v>MECHANICAL</v>
+      </c>
+      <c r="F8" s="2" t="str">
+        <v>2201 Screening</v>
+      </c>
+      <c r="G8" s="2" t="str">
+        <v>X-TT-1</v>
+      </c>
+      <c r="H8" s="2" t="str">
+        <v>Temperature transmitter</v>
+      </c>
+      <c r="I8" s="2" t="str">
+        <v>TT</v>
+      </c>
+      <c r="J8" s="2" t="str">
+        <v>X-AHU-9</v>
+      </c>
+      <c r="K8" s="2" t="str">
+        <v>VF_I&amp;C_TRANSMITTER</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="str">
+        <v>E-T2</v>
+      </c>
+      <c r="B9" s="2" t="str">
+        <v>B1</v>
+      </c>
+      <c r="C9" s="2" t="str">
+        <v>B14</v>
+      </c>
+      <c r="D9" s="2" t="str">
+        <v>2201</v>
+      </c>
+      <c r="E9" s="2" t="str">
+        <v>MECHANICAL</v>
+      </c>
+      <c r="F9" s="2" t="str">
+        <v>2201 Screening</v>
+      </c>
+      <c r="G9" s="2" t="str">
+        <v>X-TT-2</v>
+      </c>
+      <c r="H9" s="2" t="str">
+        <v>Temperature transmitter</v>
+      </c>
+      <c r="I9" s="2" t="str">
+        <v>TT</v>
+      </c>
+      <c r="J9" s="2" t="str">
+        <v>X-AHU-9</v>
+      </c>
+      <c r="K9" s="2" t="str">
+        <v>VF_I&amp;C_TRANSMITTER</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="str">
+        <v>E-T3</v>
+      </c>
+      <c r="B10" s="2" t="str">
+        <v>B1</v>
+      </c>
+      <c r="C10" s="2" t="str">
+        <v>B14</v>
+      </c>
+      <c r="D10" s="2" t="str">
+        <v>2201</v>
+      </c>
+      <c r="E10" s="2" t="str">
+        <v>MECHANICAL</v>
+      </c>
+      <c r="F10" s="2" t="str">
+        <v>2201 Screening</v>
+      </c>
+      <c r="G10" s="2" t="str">
+        <v>X-TT-3</v>
+      </c>
+      <c r="H10" s="2" t="str">
+        <v>Temperature transmitter</v>
+      </c>
+      <c r="I10" s="2" t="str">
+        <v>TT</v>
+      </c>
+      <c r="J10" s="2" t="str">
+        <v>X-AHU-9</v>
+      </c>
+      <c r="K10" s="2" t="str">
+        <v>VF_I&amp;C_TRANSMITTER</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="str">
+        <v>E-T4</v>
+      </c>
+      <c r="B11" s="2" t="str">
+        <v>B1</v>
+      </c>
+      <c r="C11" s="2" t="str">
+        <v>B14</v>
+      </c>
+      <c r="D11" s="2" t="str">
+        <v>2201</v>
+      </c>
+      <c r="E11" s="2" t="str">
+        <v>MECHANICAL</v>
+      </c>
+      <c r="F11" s="2" t="str">
+        <v>2201 Screening</v>
+      </c>
+      <c r="G11" s="2" t="str">
+        <v>X-TT-4</v>
+      </c>
+      <c r="H11" s="2" t="str">
+        <v>Temperature transmitter</v>
+      </c>
+      <c r="I11" s="2" t="str">
+        <v>TT</v>
+      </c>
+      <c r="J11" s="2" t="str">
+        <v>X-AHU-9</v>
+      </c>
+      <c r="K11" s="2" t="str">
+        <v>VF_I&amp;C_TRANSMITTER</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="str">
+        <v>E-T5</v>
+      </c>
+      <c r="B12" s="2" t="str">
+        <v>B1</v>
+      </c>
+      <c r="C12" s="2" t="str">
+        <v>B14</v>
+      </c>
+      <c r="D12" s="2" t="str">
+        <v>2201</v>
+      </c>
+      <c r="E12" s="2" t="str">
+        <v>MECHANICAL</v>
+      </c>
+      <c r="F12" s="2" t="str">
+        <v>2201 Screening</v>
+      </c>
+      <c r="G12" s="2" t="str">
+        <v>X-TT-5</v>
+      </c>
+      <c r="H12" s="2" t="str">
+        <v>Temperature transmitter</v>
+      </c>
+      <c r="I12" s="2" t="str">
+        <v>TT</v>
+      </c>
+      <c r="J12" s="2" t="str">
+        <v>X-AHU-9</v>
+      </c>
+      <c r="K12" s="2" t="str">
+        <v>VF_I&amp;C_TRANSMITTER</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="str">
+        <v>E-T6</v>
+      </c>
+      <c r="B13" s="2" t="str">
+        <v>B1</v>
+      </c>
+      <c r="C13" s="2" t="str">
+        <v>B14</v>
+      </c>
+      <c r="D13" s="2" t="str">
+        <v>2201</v>
+      </c>
+      <c r="E13" s="2" t="str">
+        <v>MECHANICAL</v>
+      </c>
+      <c r="F13" s="2" t="str">
+        <v>2201 Screening</v>
+      </c>
+      <c r="G13" s="2" t="str">
+        <v>X-TT-6</v>
+      </c>
+      <c r="H13" s="2" t="str">
+        <v>Temperature transmitter</v>
+      </c>
+      <c r="I13" s="2" t="str">
+        <v>TT</v>
+      </c>
+      <c r="J13" s="2" t="str">
+        <v>X-AHU-9</v>
+      </c>
+      <c r="K13" s="2" t="str">
+        <v>VF_I&amp;C_TRANSMITTER</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="str">
+        <v>E-T7</v>
+      </c>
+      <c r="B14" s="2" t="str">
+        <v>B1</v>
+      </c>
+      <c r="C14" s="2" t="str">
+        <v>B14</v>
+      </c>
+      <c r="D14" s="2" t="str">
+        <v>2201</v>
+      </c>
+      <c r="E14" s="2" t="str">
+        <v>MECHANICAL</v>
+      </c>
+      <c r="F14" s="2" t="str">
+        <v>2201 Screening</v>
+      </c>
+      <c r="G14" s="2" t="str">
+        <v>X-TT-7</v>
+      </c>
+      <c r="H14" s="2" t="str">
+        <v>Temperature transmitter</v>
+      </c>
+      <c r="I14" s="2" t="str">
+        <v>TT</v>
+      </c>
+      <c r="J14" s="2" t="str">
+        <v>X-AHU-9</v>
+      </c>
+      <c r="K14" s="2" t="str">
+        <v>VF_I&amp;C_TRANSMITTER</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="2" t="str">
+        <v>E-T8</v>
+      </c>
+      <c r="B15" s="2" t="str">
+        <v>B1</v>
+      </c>
+      <c r="C15" s="2" t="str">
+        <v>B14</v>
+      </c>
+      <c r="D15" s="2" t="str">
+        <v>2201</v>
+      </c>
+      <c r="E15" s="2" t="str">
+        <v>MECHANICAL</v>
+      </c>
+      <c r="F15" s="2" t="str">
+        <v>2201 Screening</v>
+      </c>
+      <c r="G15" s="2" t="str">
+        <v>X-TT-8</v>
+      </c>
+      <c r="H15" s="2" t="str">
+        <v>Temperature transmitter</v>
+      </c>
+      <c r="I15" s="2" t="str">
+        <v>TT</v>
+      </c>
+      <c r="J15" s="2" t="str">
+        <v>X-AHU-9</v>
+      </c>
+      <c r="K15" s="2" t="str">
+        <v>VF_I&amp;C_TRANSMITTER</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="2" t="str">
+        <v>E-T9</v>
+      </c>
+      <c r="B16" s="2" t="str">
+        <v>B1</v>
+      </c>
+      <c r="C16" s="2" t="str">
+        <v>B14</v>
+      </c>
+      <c r="D16" s="2" t="str">
+        <v>2201</v>
+      </c>
+      <c r="E16" s="2" t="str">
+        <v>MECHANICAL</v>
+      </c>
+      <c r="F16" s="2" t="str">
+        <v>2201 Screening</v>
+      </c>
+      <c r="G16" s="2" t="str">
+        <v>X-TT-9</v>
+      </c>
+      <c r="H16" s="2" t="str">
+        <v>Temperature transmitter</v>
+      </c>
+      <c r="I16" s="2" t="str">
+        <v>TT</v>
+      </c>
+      <c r="J16" s="2" t="str">
+        <v>X-AHU-9</v>
+      </c>
+      <c r="K16" s="2" t="str">
+        <v>VF_I&amp;C_TRANSMITTER</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="2" t="str">
         <v>E-6</v>
       </c>
-      <c r="B7" s="2" t="str">
-        <v>B1</v>
-      </c>
-      <c r="C7" s="2" t="str">
-        <v>B14</v>
-      </c>
-      <c r="D7" s="2" t="str">
+      <c r="B17" s="2" t="str">
+        <v>B1</v>
+      </c>
+      <c r="C17" s="2" t="str">
+        <v>B14</v>
+      </c>
+      <c r="D17" s="2" t="str">
         <v>266</v>
       </c>
-      <c r="E7" s="2" t="str">
+      <c r="E17" s="2" t="str">
         <v>WASTE</v>
       </c>
-      <c r="F7" s="2" t="str">
+      <c r="F17" s="2" t="str">
         <v>266 HFW Treatment</v>
       </c>
-      <c r="G7" s="2" t="str">
+      <c r="G17" s="2" t="str">
         <v>X-BLANK</v>
       </c>
-      <c r="H7" s="2" t="str">
+      <c r="H17" s="2" t="str">
         <v>Isolation valve</v>
       </c>
-      <c r="I7" s="2" t="str">
+      <c r="I17" s="2" t="str">
         <v>XV</v>
       </c>
-      <c r="J7" s="2" t="str">
+      <c r="J17" s="2" t="str">
         <v>266 HFW Treatment</v>
       </c>
-      <c r="K7" s="2" t="str">
+      <c r="K17" s="2" t="str">
         <v>VF_Blank</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:K7"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:K17"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
feat: self-graded nesting claims, flow-view controls refs, MEL-only builds
</commit_message>
<xml_diff>
--- a/tests/fixtures/compiler-extoreg.xlsx
+++ b/tests/fixtures/compiler-extoreg.xlsx
@@ -409,7 +409,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:K17"/>
+  <dimension ref="A1:K30"/>
   <sheetData>
     <row r="1">
       <c r="A1" s="2" t="str">
@@ -641,7 +641,7 @@
         <v>2201 Screening</v>
       </c>
       <c r="G7" s="2" t="str">
-        <v>X-TT-0</v>
+        <v>X-TT-9-0</v>
       </c>
       <c r="H7" s="2" t="str">
         <v>Temperature transmitter</v>
@@ -676,7 +676,7 @@
         <v>2201 Screening</v>
       </c>
       <c r="G8" s="2" t="str">
-        <v>X-TT-1</v>
+        <v>X-TT-9-1</v>
       </c>
       <c r="H8" s="2" t="str">
         <v>Temperature transmitter</v>
@@ -711,7 +711,7 @@
         <v>2201 Screening</v>
       </c>
       <c r="G9" s="2" t="str">
-        <v>X-TT-2</v>
+        <v>X-TT-9-2</v>
       </c>
       <c r="H9" s="2" t="str">
         <v>Temperature transmitter</v>
@@ -746,7 +746,7 @@
         <v>2201 Screening</v>
       </c>
       <c r="G10" s="2" t="str">
-        <v>X-TT-3</v>
+        <v>X-TT-9-3</v>
       </c>
       <c r="H10" s="2" t="str">
         <v>Temperature transmitter</v>
@@ -781,7 +781,7 @@
         <v>2201 Screening</v>
       </c>
       <c r="G11" s="2" t="str">
-        <v>X-TT-4</v>
+        <v>X-TT-9-4</v>
       </c>
       <c r="H11" s="2" t="str">
         <v>Temperature transmitter</v>
@@ -816,7 +816,7 @@
         <v>2201 Screening</v>
       </c>
       <c r="G12" s="2" t="str">
-        <v>X-TT-5</v>
+        <v>X-TT-9-5</v>
       </c>
       <c r="H12" s="2" t="str">
         <v>Temperature transmitter</v>
@@ -851,7 +851,7 @@
         <v>2201 Screening</v>
       </c>
       <c r="G13" s="2" t="str">
-        <v>X-TT-6</v>
+        <v>X-TT-9-6</v>
       </c>
       <c r="H13" s="2" t="str">
         <v>Temperature transmitter</v>
@@ -886,7 +886,7 @@
         <v>2201 Screening</v>
       </c>
       <c r="G14" s="2" t="str">
-        <v>X-TT-7</v>
+        <v>X-TT-9-7</v>
       </c>
       <c r="H14" s="2" t="str">
         <v>Temperature transmitter</v>
@@ -921,7 +921,7 @@
         <v>2201 Screening</v>
       </c>
       <c r="G15" s="2" t="str">
-        <v>X-TT-8</v>
+        <v>X-TT-9-8</v>
       </c>
       <c r="H15" s="2" t="str">
         <v>Temperature transmitter</v>
@@ -956,7 +956,7 @@
         <v>2201 Screening</v>
       </c>
       <c r="G16" s="2" t="str">
-        <v>X-TT-9</v>
+        <v>X-TT-9-9</v>
       </c>
       <c r="H16" s="2" t="str">
         <v>Temperature transmitter</v>
@@ -973,42 +973,497 @@
     </row>
     <row r="17">
       <c r="A17" s="2" t="str">
+        <v>E-P0</v>
+      </c>
+      <c r="B17" s="2" t="str">
+        <v>B1</v>
+      </c>
+      <c r="C17" s="2" t="str">
+        <v>B14</v>
+      </c>
+      <c r="D17" s="2" t="str">
+        <v>2201</v>
+      </c>
+      <c r="E17" s="2" t="str">
+        <v>MECHANICAL</v>
+      </c>
+      <c r="F17" s="2" t="str">
+        <v>2201 Screening</v>
+      </c>
+      <c r="G17" s="2" t="str">
+        <v>X-PMP-1</v>
+      </c>
+      <c r="H17" s="2" t="str">
+        <v>Screening pump</v>
+      </c>
+      <c r="I17" s="2" t="str">
+        <v>PMP</v>
+      </c>
+      <c r="J17" s="2" t="str">
+        <v>2201 Screening</v>
+      </c>
+      <c r="K17" s="2" t="str">
+        <v>VF_MECH_PUMP</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="2" t="str">
+        <v>E-P1</v>
+      </c>
+      <c r="B18" s="2" t="str">
+        <v>B1</v>
+      </c>
+      <c r="C18" s="2" t="str">
+        <v>B14</v>
+      </c>
+      <c r="D18" s="2" t="str">
+        <v>2201</v>
+      </c>
+      <c r="E18" s="2" t="str">
+        <v>MECHANICAL</v>
+      </c>
+      <c r="F18" s="2" t="str">
+        <v>2201 Screening</v>
+      </c>
+      <c r="G18" s="2" t="str">
+        <v>X-PT-9-1</v>
+      </c>
+      <c r="H18" s="2" t="str">
+        <v>Pressure transmitter</v>
+      </c>
+      <c r="I18" s="2" t="str">
+        <v>PT</v>
+      </c>
+      <c r="J18" s="2" t="str">
+        <v>X-PMP-1</v>
+      </c>
+      <c r="K18" s="2" t="str">
+        <v>VF_I&amp;C_TRANSMITTER</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="2" t="str">
+        <v>E-P2</v>
+      </c>
+      <c r="B19" s="2" t="str">
+        <v>B1</v>
+      </c>
+      <c r="C19" s="2" t="str">
+        <v>B14</v>
+      </c>
+      <c r="D19" s="2" t="str">
+        <v>2201</v>
+      </c>
+      <c r="E19" s="2" t="str">
+        <v>MECHANICAL</v>
+      </c>
+      <c r="F19" s="2" t="str">
+        <v>2201 Screening</v>
+      </c>
+      <c r="G19" s="2" t="str">
+        <v>X-PT-9-2</v>
+      </c>
+      <c r="H19" s="2" t="str">
+        <v>Pressure transmitter</v>
+      </c>
+      <c r="I19" s="2" t="str">
+        <v>PT</v>
+      </c>
+      <c r="J19" s="2" t="str">
+        <v>X-AHU-9</v>
+      </c>
+      <c r="K19" s="2" t="str">
+        <v>VF_I&amp;C_TRANSMITTER</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="2" t="str">
+        <v>E-P3</v>
+      </c>
+      <c r="B20" s="2" t="str">
+        <v>B1</v>
+      </c>
+      <c r="C20" s="2" t="str">
+        <v>B14</v>
+      </c>
+      <c r="D20" s="2" t="str">
+        <v>2201</v>
+      </c>
+      <c r="E20" s="2" t="str">
+        <v>MECHANICAL</v>
+      </c>
+      <c r="F20" s="2" t="str">
+        <v>2201 Screening</v>
+      </c>
+      <c r="G20" s="2" t="str">
+        <v>X-PT-9-3</v>
+      </c>
+      <c r="H20" s="2" t="str">
+        <v>Pressure transmitter</v>
+      </c>
+      <c r="I20" s="2" t="str">
+        <v>PT</v>
+      </c>
+      <c r="J20" s="2" t="str">
+        <v>X-PMP-1</v>
+      </c>
+      <c r="K20" s="2" t="str">
+        <v>VF_I&amp;C_TRANSMITTER</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="2" t="str">
+        <v>E-P4</v>
+      </c>
+      <c r="B21" s="2" t="str">
+        <v>B1</v>
+      </c>
+      <c r="C21" s="2" t="str">
+        <v>B14</v>
+      </c>
+      <c r="D21" s="2" t="str">
+        <v>2201</v>
+      </c>
+      <c r="E21" s="2" t="str">
+        <v>MECHANICAL</v>
+      </c>
+      <c r="F21" s="2" t="str">
+        <v>2201 Screening</v>
+      </c>
+      <c r="G21" s="2" t="str">
+        <v>X-PT-9-4</v>
+      </c>
+      <c r="H21" s="2" t="str">
+        <v>Pressure transmitter</v>
+      </c>
+      <c r="I21" s="2" t="str">
+        <v>PT</v>
+      </c>
+      <c r="J21" s="2" t="str">
+        <v>X-AHU-9</v>
+      </c>
+      <c r="K21" s="2" t="str">
+        <v>VF_I&amp;C_TRANSMITTER</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="2" t="str">
+        <v>E-P5</v>
+      </c>
+      <c r="B22" s="2" t="str">
+        <v>B1</v>
+      </c>
+      <c r="C22" s="2" t="str">
+        <v>B14</v>
+      </c>
+      <c r="D22" s="2" t="str">
+        <v>2201</v>
+      </c>
+      <c r="E22" s="2" t="str">
+        <v>MECHANICAL</v>
+      </c>
+      <c r="F22" s="2" t="str">
+        <v>2201 Screening</v>
+      </c>
+      <c r="G22" s="2" t="str">
+        <v>X-PT-9-5</v>
+      </c>
+      <c r="H22" s="2" t="str">
+        <v>Pressure transmitter</v>
+      </c>
+      <c r="I22" s="2" t="str">
+        <v>PT</v>
+      </c>
+      <c r="J22" s="2" t="str">
+        <v>X-PMP-1</v>
+      </c>
+      <c r="K22" s="2" t="str">
+        <v>VF_I&amp;C_TRANSMITTER</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="2" t="str">
+        <v>E-P6</v>
+      </c>
+      <c r="B23" s="2" t="str">
+        <v>B1</v>
+      </c>
+      <c r="C23" s="2" t="str">
+        <v>B14</v>
+      </c>
+      <c r="D23" s="2" t="str">
+        <v>2201</v>
+      </c>
+      <c r="E23" s="2" t="str">
+        <v>MECHANICAL</v>
+      </c>
+      <c r="F23" s="2" t="str">
+        <v>2201 Screening</v>
+      </c>
+      <c r="G23" s="2" t="str">
+        <v>X-PT-9-6</v>
+      </c>
+      <c r="H23" s="2" t="str">
+        <v>Pressure transmitter</v>
+      </c>
+      <c r="I23" s="2" t="str">
+        <v>PT</v>
+      </c>
+      <c r="J23" s="2" t="str">
+        <v>X-AHU-9</v>
+      </c>
+      <c r="K23" s="2" t="str">
+        <v>VF_I&amp;C_TRANSMITTER</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="2" t="str">
+        <v>E-P7</v>
+      </c>
+      <c r="B24" s="2" t="str">
+        <v>B1</v>
+      </c>
+      <c r="C24" s="2" t="str">
+        <v>B14</v>
+      </c>
+      <c r="D24" s="2" t="str">
+        <v>2201</v>
+      </c>
+      <c r="E24" s="2" t="str">
+        <v>MECHANICAL</v>
+      </c>
+      <c r="F24" s="2" t="str">
+        <v>2201 Screening</v>
+      </c>
+      <c r="G24" s="2" t="str">
+        <v>X-PT-9-7</v>
+      </c>
+      <c r="H24" s="2" t="str">
+        <v>Pressure transmitter</v>
+      </c>
+      <c r="I24" s="2" t="str">
+        <v>PT</v>
+      </c>
+      <c r="J24" s="2" t="str">
+        <v>X-PMP-1</v>
+      </c>
+      <c r="K24" s="2" t="str">
+        <v>VF_I&amp;C_TRANSMITTER</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="2" t="str">
+        <v>E-P8</v>
+      </c>
+      <c r="B25" s="2" t="str">
+        <v>B1</v>
+      </c>
+      <c r="C25" s="2" t="str">
+        <v>B14</v>
+      </c>
+      <c r="D25" s="2" t="str">
+        <v>2201</v>
+      </c>
+      <c r="E25" s="2" t="str">
+        <v>MECHANICAL</v>
+      </c>
+      <c r="F25" s="2" t="str">
+        <v>2201 Screening</v>
+      </c>
+      <c r="G25" s="2" t="str">
+        <v>X-PT-9-8</v>
+      </c>
+      <c r="H25" s="2" t="str">
+        <v>Pressure transmitter</v>
+      </c>
+      <c r="I25" s="2" t="str">
+        <v>PT</v>
+      </c>
+      <c r="J25" s="2" t="str">
+        <v>X-AHU-9</v>
+      </c>
+      <c r="K25" s="2" t="str">
+        <v>VF_I&amp;C_TRANSMITTER</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="2" t="str">
+        <v>E-P9</v>
+      </c>
+      <c r="B26" s="2" t="str">
+        <v>B1</v>
+      </c>
+      <c r="C26" s="2" t="str">
+        <v>B14</v>
+      </c>
+      <c r="D26" s="2" t="str">
+        <v>2201</v>
+      </c>
+      <c r="E26" s="2" t="str">
+        <v>MECHANICAL</v>
+      </c>
+      <c r="F26" s="2" t="str">
+        <v>2201 Screening</v>
+      </c>
+      <c r="G26" s="2" t="str">
+        <v>X-PT-9-9</v>
+      </c>
+      <c r="H26" s="2" t="str">
+        <v>Pressure transmitter</v>
+      </c>
+      <c r="I26" s="2" t="str">
+        <v>PT</v>
+      </c>
+      <c r="J26" s="2" t="str">
+        <v>X-PMP-1</v>
+      </c>
+      <c r="K26" s="2" t="str">
+        <v>VF_I&amp;C_TRANSMITTER</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="2" t="str">
+        <v>E-P10</v>
+      </c>
+      <c r="B27" s="2" t="str">
+        <v>B1</v>
+      </c>
+      <c r="C27" s="2" t="str">
+        <v>B14</v>
+      </c>
+      <c r="D27" s="2" t="str">
+        <v>2201</v>
+      </c>
+      <c r="E27" s="2" t="str">
+        <v>MECHANICAL</v>
+      </c>
+      <c r="F27" s="2" t="str">
+        <v>2201 Screening</v>
+      </c>
+      <c r="G27" s="2" t="str">
+        <v>X-PT-9-10</v>
+      </c>
+      <c r="H27" s="2" t="str">
+        <v>Pressure transmitter</v>
+      </c>
+      <c r="I27" s="2" t="str">
+        <v>PT</v>
+      </c>
+      <c r="J27" s="2" t="str">
+        <v>X-AHU-9</v>
+      </c>
+      <c r="K27" s="2" t="str">
+        <v>VF_I&amp;C_TRANSMITTER</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="2" t="str">
+        <v>E-P11</v>
+      </c>
+      <c r="B28" s="2" t="str">
+        <v>B1</v>
+      </c>
+      <c r="C28" s="2" t="str">
+        <v>B14</v>
+      </c>
+      <c r="D28" s="2" t="str">
+        <v>2201</v>
+      </c>
+      <c r="E28" s="2" t="str">
+        <v>MECHANICAL</v>
+      </c>
+      <c r="F28" s="2" t="str">
+        <v>2201 Screening</v>
+      </c>
+      <c r="G28" s="2" t="str">
+        <v>X-PT-9-11</v>
+      </c>
+      <c r="H28" s="2" t="str">
+        <v>Pressure transmitter</v>
+      </c>
+      <c r="I28" s="2" t="str">
+        <v>PT</v>
+      </c>
+      <c r="J28" s="2" t="str">
+        <v>X-PMP-1</v>
+      </c>
+      <c r="K28" s="2" t="str">
+        <v>VF_I&amp;C_TRANSMITTER</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="2" t="str">
+        <v>E-P12</v>
+      </c>
+      <c r="B29" s="2" t="str">
+        <v>B1</v>
+      </c>
+      <c r="C29" s="2" t="str">
+        <v>B14</v>
+      </c>
+      <c r="D29" s="2" t="str">
+        <v>2201</v>
+      </c>
+      <c r="E29" s="2" t="str">
+        <v>MECHANICAL</v>
+      </c>
+      <c r="F29" s="2" t="str">
+        <v>2201 Screening</v>
+      </c>
+      <c r="G29" s="2" t="str">
+        <v>X-PT-9-12</v>
+      </c>
+      <c r="H29" s="2" t="str">
+        <v>Pressure transmitter</v>
+      </c>
+      <c r="I29" s="2" t="str">
+        <v>PT</v>
+      </c>
+      <c r="J29" s="2" t="str">
+        <v>X-AHU-9</v>
+      </c>
+      <c r="K29" s="2" t="str">
+        <v>VF_I&amp;C_TRANSMITTER</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="2" t="str">
         <v>E-6</v>
       </c>
-      <c r="B17" s="2" t="str">
-        <v>B1</v>
-      </c>
-      <c r="C17" s="2" t="str">
-        <v>B14</v>
-      </c>
-      <c r="D17" s="2" t="str">
+      <c r="B30" s="2" t="str">
+        <v>B1</v>
+      </c>
+      <c r="C30" s="2" t="str">
+        <v>B14</v>
+      </c>
+      <c r="D30" s="2" t="str">
         <v>266</v>
       </c>
-      <c r="E17" s="2" t="str">
+      <c r="E30" s="2" t="str">
         <v>WASTE</v>
       </c>
-      <c r="F17" s="2" t="str">
+      <c r="F30" s="2" t="str">
         <v>266 HFW Treatment</v>
       </c>
-      <c r="G17" s="2" t="str">
+      <c r="G30" s="2" t="str">
         <v>X-BLANK</v>
       </c>
-      <c r="H17" s="2" t="str">
+      <c r="H30" s="2" t="str">
         <v>Isolation valve</v>
       </c>
-      <c r="I17" s="2" t="str">
+      <c r="I30" s="2" t="str">
         <v>XV</v>
       </c>
-      <c r="J17" s="2" t="str">
+      <c r="J30" s="2" t="str">
         <v>266 HFW Treatment</v>
       </c>
-      <c r="K17" s="2" t="str">
+      <c r="K30" s="2" t="str">
         <v>VF_Blank</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:K17"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:K30"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>